<commit_message>
Add autonomy estimation & Remove unused pictures
</commit_message>
<xml_diff>
--- a/docs/assets/images/Manufacturing/Bill of material.xlsx
+++ b/docs/assets/images/Manufacturing/Bill of material.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\btenaud\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\btenaud\Documents\02 - Projet Antenne-Terrier\02 - Git\rfid_m0.wiki\docs\assets\images\Manufacturing\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -614,9 +614,6 @@
     <t>Rocker Switch On-Off SPST Non Illuminated Panel Mount Black</t>
   </si>
   <si>
-    <t>Li-ion battery 3,6V 20Ah</t>
-  </si>
-  <si>
     <t>LiFe BATTERIES</t>
   </si>
   <si>
@@ -633,6 +630,9 @@
   </si>
   <si>
     <t>3D print ASA black</t>
+  </si>
+  <si>
+    <t>Li-ion battery 3,6V 20,8 Ah</t>
   </si>
 </sst>
 </file>
@@ -714,22 +714,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1922,10 +1907,10 @@
         <v>82</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D46" s="3">
         <v>1</v>
@@ -1942,10 +1927,10 @@
         <v>82</v>
       </c>
       <c r="B47" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="C47" s="1" t="s">
         <v>198</v>
-      </c>
-      <c r="C47" s="1" t="s">
-        <v>199</v>
       </c>
       <c r="D47" s="3">
         <v>1</v>
@@ -2319,10 +2304,10 @@
         <v>150</v>
       </c>
       <c r="B65" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="C65" s="1" t="s">
         <v>200</v>
-      </c>
-      <c r="C65" s="1" t="s">
-        <v>201</v>
       </c>
       <c r="D65" s="3">
         <v>1</v>
@@ -2593,13 +2578,13 @@
         <v>185</v>
       </c>
       <c r="C78" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="D78" s="3">
+        <v>1</v>
+      </c>
+      <c r="E78" s="10" t="s">
         <v>195</v>
-      </c>
-      <c r="D78" s="3">
-        <v>1</v>
-      </c>
-      <c r="E78" s="10" t="s">
-        <v>196</v>
       </c>
       <c r="F78" s="10" t="s">
         <v>7</v>
@@ -2621,7 +2606,7 @@
       <c r="E79" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="F79" t="s">
+      <c r="F79" s="4" t="s">
         <v>193</v>
       </c>
     </row>

</xml_diff>